<commit_message>
Ueberschuss fuer Abwaerme- und Umweltwaermebus, Zinssatz 8 Prozent, Holzverbrennungsanlagen ohne fix=Baseload-Zeitreihe, Excess District Heatbus ohne Kosten
</commit_message>
<xml_diff>
--- a/dumps/Auswertung Windpotential neu.xlsx
+++ b/dumps/Auswertung Windpotential neu.xlsx
@@ -27,12 +27,16 @@
     <sheet name="Heatpump_water" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Heatpump_recovery" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Biomasse_heat" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Biomasse_elec_heat" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Biomasse_elec_heat MWel" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="GuD" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="Biomasse_elec" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="Gesamtkosten" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="Bio feedin existing" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="Bio feedin new" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="BtL" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Fuelcell" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="PtL" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Methanisation" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,7 +502,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17347.18709266344</v>
+        <v>17410</v>
       </c>
     </row>
     <row r="6">
@@ -508,7 +512,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16670.55813098704</v>
+        <v>17410</v>
       </c>
     </row>
     <row r="7">
@@ -518,7 +522,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15949.57672401655</v>
+        <v>17410</v>
       </c>
     </row>
     <row r="8">
@@ -528,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15991.27455519061</v>
+        <v>17199.30142377931</v>
       </c>
     </row>
     <row r="9">
@@ -538,7 +542,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15954.90909293624</v>
+        <v>17060.1741740987</v>
       </c>
     </row>
     <row r="10">
@@ -548,7 +552,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15933.98004090019</v>
+        <v>17115.17108852098</v>
       </c>
     </row>
     <row r="11">
@@ -558,7 +562,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15674.65456548457</v>
+        <v>17042.36361706502</v>
       </c>
     </row>
     <row r="12">
@@ -568,7 +572,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15380.16404890747</v>
+        <v>16901.31698362184</v>
       </c>
     </row>
   </sheetData>
@@ -600,7 +604,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>207878.9587300291</v>
+        <v>991923.0162937776</v>
       </c>
     </row>
     <row r="3">
@@ -610,7 +614,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>202717.8358145564</v>
+        <v>1161233.421617127</v>
       </c>
     </row>
     <row r="4">
@@ -620,7 +624,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>206130.6060192168</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="5">
@@ -630,7 +634,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>234193.5421762202</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="6">
@@ -640,7 +644,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>279639.9975232626</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="7">
@@ -650,7 +654,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>291289.1341245184</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="8">
@@ -660,7 +664,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>680092.9465100141</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="9">
@@ -670,7 +674,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>962099.5121544122</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="10">
@@ -680,7 +684,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1193307.338080263</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="11">
@@ -690,7 +694,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1246392.494625403</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="12">
@@ -700,7 +704,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1221056.776691529</v>
+        <v>1255000</v>
       </c>
     </row>
   </sheetData>
@@ -732,7 +736,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>500000</v>
+        <v>8410.510250360863</v>
       </c>
     </row>
     <row r="3">
@@ -742,7 +746,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>500000</v>
+        <v>8911.98522417063</v>
       </c>
     </row>
     <row r="4">
@@ -752,7 +756,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>500000</v>
+        <v>9815.343017200856</v>
       </c>
     </row>
     <row r="5">
@@ -762,7 +766,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>500000</v>
+        <v>10588.1732672976</v>
       </c>
     </row>
     <row r="6">
@@ -772,7 +776,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>500000</v>
+        <v>9956.815047942411</v>
       </c>
     </row>
     <row r="7">
@@ -782,7 +786,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>500000</v>
+        <v>9266.054957153192</v>
       </c>
     </row>
     <row r="8">
@@ -792,7 +796,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>500000</v>
+        <v>9094.942509324172</v>
       </c>
     </row>
     <row r="9">
@@ -802,7 +806,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>500000</v>
+        <v>9151.511118689323</v>
       </c>
     </row>
     <row r="10">
@@ -812,7 +816,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>500000</v>
+        <v>9219.184206232267</v>
       </c>
     </row>
     <row r="11">
@@ -822,7 +826,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>500000</v>
+        <v>9232.674227619258</v>
       </c>
     </row>
     <row r="12">
@@ -832,7 +836,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>500000</v>
+        <v>9293.528427529931</v>
       </c>
     </row>
   </sheetData>
@@ -864,7 +868,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10633572.35369089</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -874,7 +878,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10691823.05805267</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -884,7 +888,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10627621.25500071</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -894,7 +898,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10525735.94077186</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -904,7 +908,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10321772.38571188</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -914,7 +918,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10118520.83446657</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -924,7 +928,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10106969.66253807</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -934,7 +938,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10100352.03139783</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -944,7 +948,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10088618.12520166</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -954,7 +958,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10045188.15293444</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -964,7 +968,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9995628.710220862</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1128,7 +1132,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3857942.749584329</v>
+        <v>3899546.649867476</v>
       </c>
     </row>
     <row r="3">
@@ -1138,7 +1142,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3190619.634492913</v>
+        <v>3927773.089776116</v>
       </c>
     </row>
     <row r="4">
@@ -1148,7 +1152,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3458251.133349622</v>
+        <v>4609164.374191121</v>
       </c>
     </row>
     <row r="5">
@@ -1158,7 +1162,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4476938.333279991</v>
+        <v>5998363.191708796</v>
       </c>
     </row>
     <row r="6">
@@ -1168,7 +1172,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5444895.671419763</v>
+        <v>7614936.100152669</v>
       </c>
     </row>
     <row r="7">
@@ -1178,7 +1182,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6576453.147613969</v>
+        <v>8985060.890569076</v>
       </c>
     </row>
     <row r="8">
@@ -1188,7 +1192,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7890334.334228567</v>
+        <v>10532308.44221447</v>
       </c>
     </row>
     <row r="9">
@@ -1198,7 +1202,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9425080.935869858</v>
+        <v>12287594.98983181</v>
       </c>
     </row>
     <row r="10">
@@ -1208,7 +1212,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11092922.57830532</v>
+        <v>14055574.49144136</v>
       </c>
     </row>
     <row r="11">
@@ -1218,7 +1222,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12919807.50779482</v>
+        <v>15794765.60923048</v>
       </c>
     </row>
     <row r="12">
@@ -1228,7 +1232,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>14860023.92295956</v>
+        <v>17601447.29623021</v>
       </c>
     </row>
   </sheetData>
@@ -1260,7 +1264,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>531.881705420592</v>
+        <v>1145.999397567335</v>
       </c>
     </row>
     <row r="3">
@@ -1270,7 +1274,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>531.495634951644</v>
+        <v>1278.615051458892</v>
       </c>
     </row>
     <row r="4">
@@ -1280,7 +1284,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>531.495634951644</v>
+        <v>1355.555156203491</v>
       </c>
     </row>
     <row r="5">
@@ -1290,7 +1294,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>552.4931125218618</v>
+        <v>1362.282381891441</v>
       </c>
     </row>
     <row r="6">
@@ -1300,7 +1304,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>577.1274858140546</v>
+        <v>1362.290407319379</v>
       </c>
     </row>
     <row r="7">
@@ -1310,7 +1314,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>586.251897658071</v>
+        <v>1510.646377848973</v>
       </c>
     </row>
     <row r="8">
@@ -1320,7 +1324,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>890.7900134139226</v>
+        <v>1623.511516749725</v>
       </c>
     </row>
     <row r="9">
@@ -1330,7 +1334,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1111.772236199733</v>
+        <v>1703.734737906207</v>
       </c>
     </row>
     <row r="10">
@@ -1340,7 +1344,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1293.842413706991</v>
+        <v>1819.411288886311</v>
       </c>
     </row>
     <row r="11">
@@ -1350,7 +1354,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1334.450220433297</v>
+        <v>1931.448186981677</v>
       </c>
     </row>
     <row r="12">
@@ -1360,7 +1364,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1315.577698904192</v>
+        <v>2016.88474764156</v>
       </c>
     </row>
   </sheetData>
@@ -1422,7 +1426,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>91.68150804318699</v>
       </c>
     </row>
     <row r="6">
@@ -1432,7 +1436,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>155.7522447752417</v>
       </c>
     </row>
     <row r="7">
@@ -1442,7 +1446,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>268.1668083954536</v>
       </c>
     </row>
     <row r="8">
@@ -1452,7 +1456,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>342.7630469820935</v>
       </c>
     </row>
     <row r="9">
@@ -1462,7 +1466,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>384.0631070789634</v>
       </c>
     </row>
     <row r="10">
@@ -1472,7 +1476,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>428.7704714064758</v>
       </c>
     </row>
     <row r="11">
@@ -1482,7 +1486,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>473.4128774115145</v>
       </c>
     </row>
     <row r="12">
@@ -1492,7 +1496,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>522.8407884633347</v>
       </c>
     </row>
   </sheetData>
@@ -1656,7 +1660,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1666,7 +1670,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1676,7 +1680,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1686,7 +1690,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1696,7 +1700,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1706,7 +1710,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1716,7 +1720,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1726,7 +1730,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1736,7 +1740,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1746,7 +1750,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1756,7 +1760,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>932.6816999999999</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1788,7 +1792,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1798,7 +1802,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1808,7 +1812,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1818,7 +1822,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1828,7 +1832,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1838,7 +1842,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1848,7 +1852,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1858,7 +1862,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1868,7 +1872,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1878,7 +1882,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1888,7 +1892,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>479.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1920,7 +1924,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3803.678886251334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1930,7 +1934,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1116.998245918806</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2184,7 +2188,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1080.296323339233</v>
       </c>
     </row>
     <row r="3">
@@ -2194,7 +2198,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>624.7852980952708</v>
       </c>
     </row>
     <row r="4">
@@ -2204,7 +2208,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>343.329103591737</v>
       </c>
     </row>
     <row r="5">
@@ -2214,7 +2218,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>293.5236035825523</v>
       </c>
     </row>
     <row r="6">
@@ -2224,7 +2228,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>294.511056438396</v>
       </c>
     </row>
     <row r="7">
@@ -2234,7 +2238,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>305.9782227262043</v>
       </c>
     </row>
     <row r="8">
@@ -2244,7 +2248,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>306.5074937820332</v>
       </c>
     </row>
     <row r="9">
@@ -2254,7 +2258,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>302.9826446808873</v>
       </c>
     </row>
     <row r="10">
@@ -2264,7 +2268,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>301.4334134873685</v>
       </c>
     </row>
     <row r="11">
@@ -2274,7 +2278,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>296.6753242540542</v>
       </c>
     </row>
     <row r="12">
@@ -2284,7 +2288,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>294.5082033537504</v>
       </c>
     </row>
   </sheetData>
@@ -2316,7 +2320,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>327.6479108166195</v>
       </c>
     </row>
     <row r="3">
@@ -2326,7 +2330,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>335.9056007305944</v>
       </c>
     </row>
     <row r="4">
@@ -2336,7 +2340,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>368.1484762682045</v>
       </c>
     </row>
     <row r="5">
@@ -2346,7 +2350,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>392.2320769914622</v>
       </c>
     </row>
     <row r="6">
@@ -2356,7 +2360,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>280.486831440746</v>
       </c>
     </row>
     <row r="7">
@@ -2366,7 +2370,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>162.9745288593218</v>
       </c>
     </row>
     <row r="8">
@@ -2376,7 +2380,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>150.7797097456288</v>
       </c>
     </row>
     <row r="9">
@@ -2386,7 +2390,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>138.1487262993318</v>
       </c>
     </row>
     <row r="10">
@@ -2396,7 +2400,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>138.6983449494151</v>
       </c>
     </row>
     <row r="11">
@@ -2406,7 +2410,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>137.3618248606762</v>
       </c>
     </row>
     <row r="12">
@@ -2416,7 +2420,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>136.8861617054585</v>
       </c>
     </row>
   </sheetData>
@@ -2580,7 +2584,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5277867053.269577</v>
+        <v>3347657152.653663</v>
       </c>
     </row>
     <row r="3">
@@ -2590,7 +2594,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4999783279.254175</v>
+        <v>3255295517.493851</v>
       </c>
     </row>
     <row r="4">
@@ -2600,7 +2604,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4779136731.196882</v>
+        <v>3137195899.46944</v>
       </c>
     </row>
     <row r="5">
@@ -2610,7 +2614,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4637433898.620055</v>
+        <v>2992177205.802913</v>
       </c>
     </row>
     <row r="6">
@@ -2620,7 +2624,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4548133199.248677</v>
+        <v>2899158706.819975</v>
       </c>
     </row>
     <row r="7">
@@ -2630,7 +2634,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4485755287.912626</v>
+        <v>2825657321.700679</v>
       </c>
     </row>
     <row r="8">
@@ -2640,7 +2644,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4424064438.323107</v>
+        <v>2731745568.856122</v>
       </c>
     </row>
     <row r="9">
@@ -2650,7 +2654,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4371855469.58036</v>
+        <v>2628100409.656794</v>
       </c>
     </row>
     <row r="10">
@@ -2660,7 +2664,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4321066743.952408</v>
+        <v>2570123617.255716</v>
       </c>
     </row>
     <row r="11">
@@ -2670,7 +2674,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4279503861.095598</v>
+        <v>2512686004.332447</v>
       </c>
     </row>
     <row r="12">
@@ -2680,7 +2684,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4239220808.454051</v>
+        <v>2465973974.958939</v>
       </c>
     </row>
   </sheetData>
@@ -2712,7 +2716,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>258.2563557551648</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3">
@@ -2722,7 +2726,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>258.2563557551638</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4">
@@ -2732,7 +2736,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>258.2563557551525</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5">
@@ -2742,7 +2746,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>258.256355755162</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6">
@@ -2752,7 +2756,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>258.2563557551561</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7">
@@ -2762,7 +2766,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>258.2563557551564</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8">
@@ -2772,7 +2776,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>258.2563557551632</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9">
@@ -2782,7 +2786,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>258.2563557551575</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10">
@@ -2792,7 +2796,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>258.2563557551586</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11">
@@ -2802,7 +2806,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>258.2563557551581</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12">
@@ -2812,7 +2816,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>258.2563557551599</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -2844,7 +2848,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>81.37100752285787</v>
       </c>
     </row>
     <row r="3">
@@ -2854,7 +2858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>81.37100752285727</v>
       </c>
     </row>
     <row r="4">
@@ -2864,7 +2868,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>81.00183824198079</v>
       </c>
     </row>
     <row r="5">
@@ -2874,7 +2878,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>80.11087149449362</v>
       </c>
     </row>
     <row r="6">
@@ -2884,7 +2888,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>41.35569008295406</v>
       </c>
     </row>
     <row r="7">
@@ -2894,7 +2898,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>7.254993502090978</v>
       </c>
     </row>
     <row r="8">
@@ -2904,7 +2908,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>3.223921685924616</v>
       </c>
     </row>
     <row r="9">
@@ -2945,6 +2949,402 @@
       </c>
       <c r="B12" t="n">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>kein Wind</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6.10074188529427</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6.10074188529427</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6.293716736674904</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6.75944935467947</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>27.01783963796747</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>44.84320375981726</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>46.95035493643235</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>48.63558672679329</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>48.63558672679329</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>48.63558672679329</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>viel Wind</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>48.63558672679329</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>kein Wind</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>viel Wind</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>kein Wind</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>57.11704865389363</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>103.0608761479687</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>135.3949512353719</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>181.6289795574187</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>225.8014910766373</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>viel Wind</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>258.6945669306924</v>
       </c>
     </row>
   </sheetData>
@@ -3084,6 +3484,138 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>kein Wind</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>viel Wind</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3240,7 +3772,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9121315.806178465</v>
+        <v>1955671.264047959</v>
       </c>
     </row>
     <row r="3">
@@ -3250,7 +3782,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8253681.821670347</v>
+        <v>2507428.877332959</v>
       </c>
     </row>
     <row r="4">
@@ -3260,7 +3792,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7133561.776725775</v>
+        <v>2781567.830964216</v>
       </c>
     </row>
     <row r="5">
@@ -3270,7 +3802,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6027114.71874018</v>
+        <v>2437507.989503615</v>
       </c>
     </row>
     <row r="6">
@@ -3280,7 +3812,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5480964.239672538</v>
+        <v>2238717.896834248</v>
       </c>
     </row>
     <row r="7">
@@ -3290,7 +3822,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5109557.725735168</v>
+        <v>2131089.562876385</v>
       </c>
     </row>
     <row r="8">
@@ -3300,7 +3832,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4726671.175088175</v>
+        <v>2008664.060209167</v>
       </c>
     </row>
     <row r="9">
@@ -3310,7 +3842,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4427415.157965422</v>
+        <v>1897284.413970993</v>
       </c>
     </row>
     <row r="10">
@@ -3320,7 +3852,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4183752.313580773</v>
+        <v>1786728.192735474</v>
       </c>
     </row>
     <row r="11">
@@ -3330,7 +3862,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4014338.395778846</v>
+        <v>1740522.222969331</v>
       </c>
     </row>
     <row r="12">
@@ -3340,7 +3872,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3859021.215512211</v>
+        <v>1700091.47137775</v>
       </c>
     </row>
   </sheetData>
@@ -3372,7 +3904,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5000</v>
+        <v>2220.167595875623</v>
       </c>
     </row>
     <row r="3">
@@ -3636,7 +4168,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9092.98738875538</v>
+        <v>5340.353221551798</v>
       </c>
     </row>
     <row r="3">
@@ -3646,7 +4178,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6951.952531039873</v>
+        <v>5417.921583967126</v>
       </c>
     </row>
     <row r="4">
@@ -3656,7 +4188,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5538.030925930791</v>
+        <v>5850.558190201666</v>
       </c>
     </row>
     <row r="5">
@@ -3666,7 +4198,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5216.651736913682</v>
+        <v>5902.849230327291</v>
       </c>
     </row>
     <row r="6">
@@ -3676,7 +4208,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4848.974497715429</v>
+        <v>5905.922424258713</v>
       </c>
     </row>
     <row r="7">
@@ -3686,7 +4218,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4710.594848835342</v>
+        <v>5671.551242182106</v>
       </c>
     </row>
     <row r="8">
@@ -3696,7 +4228,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4697.131582531629</v>
+        <v>5509.790374575122</v>
       </c>
     </row>
     <row r="9">
@@ -3706,7 +4238,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4709.425142336809</v>
+        <v>5485.12893245917</v>
       </c>
     </row>
     <row r="10">
@@ -3716,7 +4248,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4646.966149001297</v>
+        <v>5427.746283559022</v>
       </c>
     </row>
     <row r="11">
@@ -3726,7 +4258,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4583.815148778218</v>
+        <v>5185.751100322449</v>
       </c>
     </row>
     <row r="12">
@@ -3736,7 +4268,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4593.427292030163</v>
+        <v>4955.641895930417</v>
       </c>
     </row>
   </sheetData>
@@ -3768,7 +4300,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>454294.5172354548</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="3">
@@ -3778,7 +4310,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>454294.5172354584</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="4">
@@ -3788,7 +4320,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>454294.5172354474</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="5">
@@ -3798,7 +4330,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>454294.5172354652</v>
+        <v>1094755.335599623</v>
       </c>
     </row>
     <row r="6">
@@ -3808,7 +4340,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>454294.5172354876</v>
+        <v>872308.1118757005</v>
       </c>
     </row>
     <row r="7">
@@ -3818,7 +4350,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>454294.5172354684</v>
+        <v>682778.8739722851</v>
       </c>
     </row>
     <row r="8">
@@ -3828,7 +4360,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>454294.5172354415</v>
+        <v>661996.1247681077</v>
       </c>
     </row>
     <row r="9">
@@ -3838,7 +4370,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>454294.5172354591</v>
+        <v>645405.5774503113</v>
       </c>
     </row>
     <row r="10">
@@ -3848,7 +4380,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>454294.5172354496</v>
+        <v>645405.5774503113</v>
       </c>
     </row>
     <row r="11">
@@ -3858,7 +4390,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>454294.5172354385</v>
+        <v>645405.5774503113</v>
       </c>
     </row>
     <row r="12">
@@ -3868,7 +4400,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>454294.5172354744</v>
+        <v>645405.5774503113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Waermepumpen bearbeitet, PtL Wirkungsgrad, Biomasse constraint, H2 Speicher Wirkungsgrad ausspeichern
</commit_message>
<xml_diff>
--- a/dumps/Auswertung Windpotential neu.xlsx
+++ b/dumps/Auswertung Windpotential neu.xlsx
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17199.30142377931</v>
+        <v>17410</v>
       </c>
     </row>
     <row r="9">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17060.1741740987</v>
+        <v>17410</v>
       </c>
     </row>
     <row r="10">
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17115.17108852098</v>
+        <v>17410</v>
       </c>
     </row>
     <row r="11">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17042.36361706502</v>
+        <v>17410</v>
       </c>
     </row>
     <row r="12">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16901.31698362184</v>
+        <v>17410</v>
       </c>
     </row>
   </sheetData>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>991923.0162937776</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="3">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1161233.421617127</v>
+        <v>1255000</v>
       </c>
     </row>
     <row r="4">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8410.510250360863</v>
+        <v>8394.410095388828</v>
       </c>
     </row>
     <row r="3">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8911.98522417063</v>
+        <v>8534.621727128209</v>
       </c>
     </row>
     <row r="4">
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9815.343017200856</v>
+        <v>9129.699044934237</v>
       </c>
     </row>
     <row r="5">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10588.1732672976</v>
+        <v>9553.673486214435</v>
       </c>
     </row>
     <row r="6">
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9956.815047942411</v>
+        <v>9717.867374330943</v>
       </c>
     </row>
     <row r="7">
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9266.054957153192</v>
+        <v>9894.705611385913</v>
       </c>
     </row>
     <row r="8">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9094.942509324172</v>
+        <v>12735.92761637438</v>
       </c>
     </row>
     <row r="9">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9151.511118689323</v>
+        <v>15505.17734018857</v>
       </c>
     </row>
     <row r="10">
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9219.184206232267</v>
+        <v>15621.93817988038</v>
       </c>
     </row>
     <row r="11">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9232.674227619258</v>
+        <v>14840.38330587905</v>
       </c>
     </row>
     <row r="12">
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9293.528427529931</v>
+        <v>14546.12831908544</v>
       </c>
     </row>
   </sheetData>
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3899546.649867476</v>
+        <v>2352299.931756873</v>
       </c>
     </row>
     <row r="3">
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3927773.089776116</v>
+        <v>2252622.925309703</v>
       </c>
     </row>
     <row r="4">
@@ -1152,7 +1152,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4609164.374191121</v>
+        <v>2799487.869400776</v>
       </c>
     </row>
     <row r="5">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5998363.191708796</v>
+        <v>3946592.248236736</v>
       </c>
     </row>
     <row r="6">
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7614936.100152669</v>
+        <v>5338198.427567813</v>
       </c>
     </row>
     <row r="7">
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8985060.890569076</v>
+        <v>6863073.78584145</v>
       </c>
     </row>
     <row r="8">
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10532308.44221447</v>
+        <v>8470008.874338269</v>
       </c>
     </row>
     <row r="9">
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12287594.98983181</v>
+        <v>10268757.54174227</v>
       </c>
     </row>
     <row r="10">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14055574.49144136</v>
+        <v>12277255.9222215</v>
       </c>
     </row>
     <row r="11">
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15794765.60923048</v>
+        <v>14383634.02512666</v>
       </c>
     </row>
     <row r="12">
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>17601447.29623021</v>
+        <v>16504765.50083046</v>
       </c>
     </row>
   </sheetData>
@@ -1264,7 +1264,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1145.999397567335</v>
+        <v>1686.246368756388</v>
       </c>
     </row>
     <row r="3">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1278.615051458892</v>
+        <v>1678.085546841403</v>
       </c>
     </row>
     <row r="4">
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1355.555156203491</v>
+        <v>1688.316414268532</v>
       </c>
     </row>
     <row r="5">
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1362.282381891441</v>
+        <v>1693.182256270397</v>
       </c>
     </row>
     <row r="6">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1362.290407319379</v>
+        <v>1740.140355566713</v>
       </c>
     </row>
     <row r="7">
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1510.646377848973</v>
+        <v>1827.831930581633</v>
       </c>
     </row>
     <row r="8">
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1623.511516749725</v>
+        <v>1836.672384798126</v>
       </c>
     </row>
     <row r="9">
@@ -1334,7 +1334,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1703.734737906207</v>
+        <v>1840.524696651325</v>
       </c>
     </row>
     <row r="10">
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1819.411288886311</v>
+        <v>1844.662594717072</v>
       </c>
     </row>
     <row r="11">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1931.448186981677</v>
+        <v>1844.662594717072</v>
       </c>
     </row>
     <row r="12">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2016.88474764156</v>
+        <v>1844.662594717072</v>
       </c>
     </row>
   </sheetData>
@@ -1396,7 +1396,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>343.2195891155749</v>
       </c>
     </row>
     <row r="3">
@@ -1406,7 +1406,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>336.0814781421718</v>
       </c>
     </row>
     <row r="4">
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>357.7116390902225</v>
       </c>
     </row>
     <row r="5">
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>91.68150804318699</v>
+        <v>398.0560024549026</v>
       </c>
     </row>
     <row r="6">
@@ -1436,7 +1436,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>155.7522447752417</v>
+        <v>446.2835296400118</v>
       </c>
     </row>
     <row r="7">
@@ -1446,7 +1446,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>268.1668083954536</v>
+        <v>470.465022415357</v>
       </c>
     </row>
     <row r="8">
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>342.7630469820935</v>
+        <v>706.5324839878549</v>
       </c>
     </row>
     <row r="9">
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>384.0631070789634</v>
+        <v>938.8751107559603</v>
       </c>
     </row>
     <row r="10">
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>428.7704714064758</v>
+        <v>971.7947103755469</v>
       </c>
     </row>
     <row r="11">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>473.4128774115145</v>
+        <v>950.9214920105085</v>
       </c>
     </row>
     <row r="12">
@@ -1496,7 +1496,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>522.8407884633347</v>
+        <v>944.7536962607035</v>
       </c>
     </row>
   </sheetData>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>114.9950097286183</v>
       </c>
     </row>
     <row r="3">
@@ -1538,7 +1538,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>115.4834209214472</v>
       </c>
     </row>
     <row r="4">
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>111.265026311643</v>
       </c>
     </row>
     <row r="5">
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>99.76661547501115</v>
       </c>
     </row>
     <row r="6">
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>90.33378662671147</v>
       </c>
     </row>
     <row r="7">
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>86.6885348102485</v>
       </c>
     </row>
     <row r="8">
@@ -1588,7 +1588,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>51.26258806051763</v>
       </c>
     </row>
     <row r="9">
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>18.90110190708293</v>
       </c>
     </row>
     <row r="10">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>3.750418084124513</v>
       </c>
     </row>
     <row r="11">
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2466.721630745905</v>
       </c>
     </row>
     <row r="3">
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>749.4174511065776</v>
       </c>
     </row>
     <row r="4">
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1080.296323339233</v>
+        <v>217.2515863354713</v>
       </c>
     </row>
     <row r="3">
@@ -2198,7 +2198,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>624.7852980952708</v>
+        <v>216.7685469754418</v>
       </c>
     </row>
     <row r="4">
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>343.329103591737</v>
+        <v>210.1691980130085</v>
       </c>
     </row>
     <row r="5">
@@ -2218,7 +2218,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>293.5236035825523</v>
+        <v>210.0438540207381</v>
       </c>
     </row>
     <row r="6">
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>294.511056438396</v>
+        <v>212.4913269213288</v>
       </c>
     </row>
     <row r="7">
@@ -2238,7 +2238,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>305.9782227262043</v>
+        <v>211.0390985860681</v>
       </c>
     </row>
     <row r="8">
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>306.5074937820332</v>
+        <v>216.6940984707007</v>
       </c>
     </row>
     <row r="9">
@@ -2258,7 +2258,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>302.9826446808873</v>
+        <v>220.7034562169137</v>
       </c>
     </row>
     <row r="10">
@@ -2268,7 +2268,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>301.4334134873685</v>
+        <v>222.4690754681357</v>
       </c>
     </row>
     <row r="11">
@@ -2278,7 +2278,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>296.6753242540542</v>
+        <v>222.7830188860003</v>
       </c>
     </row>
     <row r="12">
@@ -2288,7 +2288,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>294.5082033537504</v>
+        <v>221.41552574064</v>
       </c>
     </row>
   </sheetData>
@@ -2320,7 +2320,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>327.6479108166195</v>
+        <v>299.3091481644382</v>
       </c>
     </row>
     <row r="3">
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>335.9056007305944</v>
+        <v>304.1262197479463</v>
       </c>
     </row>
     <row r="4">
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>368.1484762682045</v>
+        <v>336.3601112593572</v>
       </c>
     </row>
     <row r="5">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>392.2320769914622</v>
+        <v>373.1066745048118</v>
       </c>
     </row>
     <row r="6">
@@ -2360,7 +2360,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>280.486831440746</v>
+        <v>403.9411972813725</v>
       </c>
     </row>
     <row r="7">
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>162.9745288593218</v>
+        <v>407.829566326499</v>
       </c>
     </row>
     <row r="8">
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>150.7797097456288</v>
+        <v>414.7655446945025</v>
       </c>
     </row>
     <row r="9">
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>138.1487262993318</v>
+        <v>413.9017321397615</v>
       </c>
     </row>
     <row r="10">
@@ -2400,7 +2400,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>138.6983449494151</v>
+        <v>407.0784379632078</v>
       </c>
     </row>
     <row r="11">
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>137.3618248606762</v>
+        <v>403.6020470599593</v>
       </c>
     </row>
     <row r="12">
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>136.8861617054585</v>
+        <v>396.6638350781536</v>
       </c>
     </row>
   </sheetData>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3347657152.653663</v>
+        <v>3310308933.945353</v>
       </c>
     </row>
     <row r="3">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3255295517.493851</v>
+        <v>3061936357.199508</v>
       </c>
     </row>
     <row r="4">
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3137195899.46944</v>
+        <v>2854036318.138533</v>
       </c>
     </row>
     <row r="5">
@@ -2614,7 +2614,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2992177205.802913</v>
+        <v>2702910174.233757</v>
       </c>
     </row>
     <row r="6">
@@ -2624,7 +2624,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2899158706.819975</v>
+        <v>2585580835.815068</v>
       </c>
     </row>
     <row r="7">
@@ -2634,7 +2634,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2825657321.700679</v>
+        <v>2474591240.652443</v>
       </c>
     </row>
     <row r="8">
@@ -2644,7 +2644,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2731745568.856122</v>
+        <v>2354900737.874852</v>
       </c>
     </row>
     <row r="9">
@@ -2654,7 +2654,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2628100409.656794</v>
+        <v>2240027777.819066</v>
       </c>
     </row>
     <row r="10">
@@ -2664,7 +2664,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2570123617.255716</v>
+        <v>2177999064.090259</v>
       </c>
     </row>
     <row r="11">
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2512686004.332447</v>
+        <v>2117782081.142441</v>
       </c>
     </row>
     <row r="12">
@@ -2684,7 +2684,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2465973974.958939</v>
+        <v>2058342789.262475</v>
       </c>
     </row>
   </sheetData>
@@ -2848,7 +2848,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81.37100752285787</v>
+        <v>81.37100752286068</v>
       </c>
     </row>
     <row r="3">
@@ -2858,7 +2858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81.37100752285727</v>
+        <v>81.37100752285515</v>
       </c>
     </row>
     <row r="4">
@@ -2868,7 +2868,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>81.00183824198079</v>
+        <v>81.37100752285282</v>
       </c>
     </row>
     <row r="5">
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80.11087149449362</v>
+        <v>81.37100752285284</v>
       </c>
     </row>
     <row r="6">
@@ -2888,7 +2888,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>41.35569008295406</v>
+        <v>81.37100752285279</v>
       </c>
     </row>
     <row r="7">
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.254993502090978</v>
+        <v>81.37100752285285</v>
       </c>
     </row>
     <row r="8">
@@ -2908,7 +2908,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3.223921685924616</v>
+        <v>81.37100752285289</v>
       </c>
     </row>
     <row r="9">
@@ -2918,7 +2918,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>81.37100752285284</v>
       </c>
     </row>
     <row r="10">
@@ -2928,7 +2928,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>81.37100752285458</v>
       </c>
     </row>
     <row r="11">
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>81.37100752285458</v>
       </c>
     </row>
     <row r="12">
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>81.3710075228546</v>
       </c>
     </row>
   </sheetData>
@@ -2980,7 +2980,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6.10074188529427</v>
+        <v>6.085144214328512</v>
       </c>
     </row>
     <row r="3">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.10074188529427</v>
+        <v>6.085144214338694</v>
       </c>
     </row>
     <row r="4">
@@ -3000,7 +3000,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.293716736674904</v>
+        <v>6.085144214333875</v>
       </c>
     </row>
     <row r="5">
@@ -3010,7 +3010,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.75944935467947</v>
+        <v>6.085144214333863</v>
       </c>
     </row>
     <row r="6">
@@ -3020,7 +3020,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27.01783963796747</v>
+        <v>6.08514421433382</v>
       </c>
     </row>
     <row r="7">
@@ -3030,7 +3030,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44.84320375981726</v>
+        <v>6.085144214333069</v>
       </c>
     </row>
     <row r="8">
@@ -3040,7 +3040,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>46.95035493643235</v>
+        <v>6.085144214333473</v>
       </c>
     </row>
     <row r="9">
@@ -3050,7 +3050,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>48.63558672679329</v>
+        <v>6.085144214333517</v>
       </c>
     </row>
     <row r="10">
@@ -3060,7 +3060,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>48.63558672679329</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -3070,7 +3070,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48.63558672679329</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -3080,7 +3080,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>48.63558672679329</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3244,7 +3244,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>479.4500102193472</v>
       </c>
     </row>
     <row r="3">
@@ -3254,7 +3254,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>479.4500102193371</v>
       </c>
     </row>
     <row r="4">
@@ -3264,7 +3264,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>479.4500102193419</v>
       </c>
     </row>
     <row r="5">
@@ -3274,7 +3274,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>479.4500102193419</v>
       </c>
     </row>
     <row r="6">
@@ -3284,7 +3284,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>479.4500102193419</v>
       </c>
     </row>
     <row r="7">
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>57.11704865389363</v>
+        <v>479.4500102193427</v>
       </c>
     </row>
     <row r="8">
@@ -3304,7 +3304,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>103.0608761479687</v>
+        <v>479.4500102193423</v>
       </c>
     </row>
     <row r="9">
@@ -3314,7 +3314,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>135.3949512353719</v>
+        <v>479.4500102193421</v>
       </c>
     </row>
     <row r="10">
@@ -3324,7 +3324,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>181.6289795574187</v>
+        <v>485.5351544336758</v>
       </c>
     </row>
     <row r="11">
@@ -3334,7 +3334,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>225.8014910766373</v>
+        <v>485.5351544336756</v>
       </c>
     </row>
     <row r="12">
@@ -3344,7 +3344,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>258.6945669306924</v>
+        <v>485.5351544336756</v>
       </c>
     </row>
   </sheetData>
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="3">
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="4">
@@ -3660,7 +3660,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="5">
@@ -3670,7 +3670,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="6">
@@ -3680,7 +3680,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="7">
@@ -3690,7 +3690,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="8">
@@ -3700,7 +3700,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="9">
@@ -3710,7 +3710,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="10">
@@ -3720,7 +3720,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="11">
@@ -3730,7 +3730,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
     <row r="12">
@@ -3740,7 +3740,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>0.01695399018152757</v>
       </c>
     </row>
   </sheetData>
@@ -3772,7 +3772,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1955671.264047959</v>
+        <v>6518165.818678496</v>
       </c>
     </row>
     <row r="3">
@@ -3782,7 +3782,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2507428.877332959</v>
+        <v>5475246.89775872</v>
       </c>
     </row>
     <row r="4">
@@ -3792,7 +3792,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2781567.830964216</v>
+        <v>4474267.112656175</v>
       </c>
     </row>
     <row r="5">
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2437507.989503615</v>
+        <v>3639945.150598565</v>
       </c>
     </row>
     <row r="6">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2238717.896834248</v>
+        <v>3202500.830594863</v>
       </c>
     </row>
     <row r="7">
@@ -3822,7 +3822,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2131089.562876385</v>
+        <v>2895225.414598964</v>
       </c>
     </row>
     <row r="8">
@@ -3832,7 +3832,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2008664.060209167</v>
+        <v>2631525.256123828</v>
       </c>
     </row>
     <row r="9">
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1897284.413970993</v>
+        <v>2416334.960509835</v>
       </c>
     </row>
     <row r="10">
@@ -3852,7 +3852,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1786728.192735474</v>
+        <v>2302252.949770859</v>
       </c>
     </row>
     <row r="11">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1740522.222969331</v>
+        <v>2179387.114314807</v>
       </c>
     </row>
     <row r="12">
@@ -3872,7 +3872,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1700091.47137775</v>
+        <v>2045079.919698146</v>
       </c>
     </row>
   </sheetData>
@@ -3904,7 +3904,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2220.167595875623</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
@@ -4168,7 +4168,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5340.353221551798</v>
+        <v>9881.01937634471</v>
       </c>
     </row>
     <row r="3">
@@ -4178,7 +4178,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5417.921583967126</v>
+        <v>7864.657963989617</v>
       </c>
     </row>
     <row r="4">
@@ -4188,7 +4188,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5850.558190201666</v>
+        <v>6295.322053401311</v>
       </c>
     </row>
     <row r="5">
@@ -4198,7 +4198,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5902.849230327291</v>
+        <v>6105.810483399178</v>
       </c>
     </row>
     <row r="6">
@@ -4208,7 +4208,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5905.922424258713</v>
+        <v>5868.633675515071</v>
       </c>
     </row>
     <row r="7">
@@ -4218,7 +4218,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5671.551242182106</v>
+        <v>5745.954256751552</v>
       </c>
     </row>
     <row r="8">
@@ -4228,7 +4228,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5509.790374575122</v>
+        <v>5788.911445297143</v>
       </c>
     </row>
     <row r="9">
@@ -4238,7 +4238,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5485.12893245917</v>
+        <v>5930.7092403229</v>
       </c>
     </row>
     <row r="10">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5427.746283559022</v>
+        <v>5786.827216554539</v>
       </c>
     </row>
     <row r="11">
@@ -4258,7 +4258,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5185.751100322449</v>
+        <v>5746.366348089974</v>
       </c>
     </row>
     <row r="12">
@@ -4268,7 +4268,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4955.641895930417</v>
+        <v>5880.97396394353</v>
       </c>
     </row>
   </sheetData>
@@ -4330,7 +4330,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1094755.335599623</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="6">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>872308.1118757005</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="7">
@@ -4350,7 +4350,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>682778.8739722851</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="8">
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>661996.1247681077</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="9">
@@ -4370,7 +4370,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>645405.5774503113</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="10">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>645405.5774503113</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="11">
@@ -4390,7 +4390,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>645405.5774503113</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="12">
@@ -4400,7 +4400,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>645405.5774503113</v>
+        <v>1100000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>